<commit_message>
Workbench: measured PC preflight 19-10-2026 (step A, plain run)
Verdict READY WITH CONDITIONS. Hyper-V not installed; only C: and the
AVNI OS SanDisk SSD connected, 2 TB HDD absent -> no drive chosen.
Tracker items 2, 4, 30 updated. Raw report kept on the PC (public repo).
Handshake job HS-20261019-090459.
Lease: none - not a registered AVNI mutation target (GitHub-only project).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent-workbench/TRACKER.xlsx
+++ b/agent-workbench/TRACKER.xlsx
@@ -568,7 +568,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>host/Preflight-Workbench.ps1. Parse-checked with PowerShell 7 on Linux only. CONFIGURED - UNVERIFIED until it runs on the real PC.</t>
+          <t>Plain run on the PC 19-10-2026 09:06: READY WITH CONDITIONS. Hyper-V not installed (no vmms, no module), hypervisor on (VBS). RAM 31.3/10.2 GB free -&gt; 6 GB VM. Elevated re-run waits for the Hyper-V permission. See PREFLIGHT-19-10-2026.md</t>
         </is>
       </c>
     </row>
@@ -611,9 +611,9 @@
           <t>Stage 0 - Owner decision: which drive holds the VHDX (not C:)</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>DECIDED (Architect 18-10-2026): choose only after preflight from measured, suitable fixed drives. C: untouched. The SSD reserved for AVNI OS is EXCLUDED. The 2 TB HDD is the candidate if preflight shows it healthy, with free space and acceptable performance. Never guess the letter.</t>
+          <t>Rule decided 18-10; measured 19-10: only C: (system) and E: (USB SanDisk SSD, kept for AVNI OS) are connected. 2 TB HDD absent -&gt; no drive chosen, nothing allocated</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Architect 18-10-2026: evaluate performance, not only capacity. A VHDX on a slow HDD makes the guest desktop sluggish; preflight numbers decide.</t>
+          <t>19-10-2026: 2 TB HDD not connected to the PC (Get-PhysicalDisk shows only disk 0 NVMe + disk 1 SanDisk USB). Owner to plug it in</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Workbench: PC preflight 21-10-2026 plain + elevated (step A), Hyper-V switched on (restart pending), tracker 2/4/30; 'Partial' -> 'Open' (Ravi 20-10)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent-workbench/TRACKER.xlsx
+++ b/agent-workbench/TRACKER.xlsx
@@ -553,22 +553,23 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>1 session</t>
+          <t>17 s plain + 41 s elevated</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Run on PC: next local session, 5 min</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Plain run on the PC 19-10-2026 09:06: READY WITH CONDITIONS. Hyper-V not installed (no vmms, no module), hypervisor on (VBS). RAM 31.3/10.2 GB free -&gt; 6 GB VM. Elevated re-run waits for the Hyper-V permission. See PREFLIGHT-19-10-2026.md</t>
+          <t>21-10-2026: plain run 17:49 and ELEVATED run 17:50 (UAC pressed by Ravi at the PC) - both READY WITH CONDITIONS. Measured: Microsoft-Hyper-V-All = Disabled; no Hyper-V module, no vmms; hypervisor present (VBS). RAM 63.3 GB total / 29.8 GB free -&gt; 8 GB VM. Fixed drives: C: 57.7 GB free (system, excluded), E: 845.9 GB free. Then 17:52 elevated: Enable-WindowsOptionalFeature Microsoft-Hyper-V-All -NoRestart -&gt; all 7 Hyper-V features Enabled, RestartNeeded = True (completes at the next power-off). Raw reports on the PC only: %LOCALAPPDATA%\Avni+eports\workbench-preflight-21-10-2026_1749 / _1750 and workbench-hyperv-enable-21-10-2026.log. See PREFLIGHT-21-10-2026.md</t>
         </is>
       </c>
     </row>
@@ -613,7 +614,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -628,7 +629,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Rule decided 18-10; measured 19-10: only C: (system) and E: (USB SanDisk SSD, kept for AVNI OS) are connected. 2 TB HDD absent -&gt; no drive chosen, nothing allocated</t>
+          <t>Rule decided 18-10; measured 19-10: only C: (system) and E: (USB SanDisk SSD, kept for AVNI OS) are connected. 2 TB HDD absent -&gt; no drive chosen, nothing allocated | 20-10-2026 14:38 Ravi (phone ask-33c40ae475724999): 'I will plug in the 2 TB disk and allow Hyper-V'. 21-10-2026 17:4x: Hyper-V allowed and switched on; the 2 TB disk is still not connected (only C: and E:). No drive chosen, nothing allocated.</t>
         </is>
       </c>
     </row>
@@ -643,7 +644,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -733,7 +734,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -763,7 +764,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -793,7 +794,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -853,7 +854,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -883,7 +884,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -913,7 +914,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1153,7 +1154,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1183,7 +1184,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1393,7 +1394,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1408,7 +1409,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>19-10-2026: 2 TB HDD not connected to the PC (Get-PhysicalDisk shows only disk 0 NVMe + disk 1 SanDisk USB). Owner to plug it in</t>
+          <t>19-10-2026: 2 TB HDD not connected to the PC (Get-PhysicalDisk shows only disk 0 NVMe + disk 1 SanDisk USB). Owner to plug it in | 21-10-2026 17:4x: still not connected (Get-Disk: 0 Samsung NVMe, 1 SanDisk USB).</t>
         </is>
       </c>
     </row>
@@ -1487,12 +1488,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Built, not yet verified where it must run. CONFIGURED - UNVERIFIED.</t>
+          <t>Started, not finished (Ravi 20-10-2026: the word 'partial' is not used anywhere in AVNI)</t>
         </is>
       </c>
     </row>
@@ -1544,6 +1545,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Workbench: guest hands service tests pass on Windows 21-10-2026 (54 ran, 0 failures, 4 skipped)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent-workbench/TRACKER.xlsx
+++ b/agent-workbench/TRACKER.xlsx
@@ -779,7 +779,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>guest/avni_hands.py. Pure-logic parts unit-tested on Linux; user32/SendInput path UNVERIFIED until run in the guest.</t>
+          <t>guest/avni_hands.py. Pure-logic parts unit-tested on Linux; user32/SendInput path UNVERIFIED until run in the guest. | 21-10-2026 18:09 TESTED on the PC (Windows, Python 3.14, Pillow + pywin32 installed): unittest discover guest/ -&gt; 54 ran, 0 failures, 4 skipped. Not yet installed in a guest (no VM yet).</t>
         </is>
       </c>
     </row>
@@ -809,7 +809,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>host/workbench_driver.py. Tested on Linux only against the hands service in --dry-run mode.</t>
+          <t>host/workbench_driver.py. Tested on Linux only against the hands service in --dry-run mode. | 21-10-2026 18:09 TESTED on the PC (Windows, Python 3.14, Pillow + pywin32 installed): unittest discover guest/ -&gt; 54 ran, 0 failures, 4 skipped. Not yet installed in a guest (no VM yet).</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Service now refuses every client except localhost and the default gateway (= the host on Default Switch) with 403 BEFORE the token check; --allow-client / --allow-any-client to widen on purpose. Installer firewall rule limited to -RemoteAddress &lt;gateway&gt;. 13 new unit tests pass on Linux. Token still travels over plain HTTP on the host-guest link: accepted for the pilot, noted.</t>
+          <t>Service now refuses every client except localhost and the default gateway (= the host on Default Switch) with 403 BEFORE the token check; --allow-client / --allow-any-client to widen on purpose. Installer firewall rule limited to -RemoteAddress &lt;gateway&gt;. 13 new unit tests pass on Linux. Token still travels over plain HTTP on the host-guest link: accepted for the pilot, noted. | 21-10-2026 18:09 TESTED on the PC (Windows, Python 3.14, Pillow + pywin32 installed): unittest discover guest/ -&gt; 54 ran, 0 failures, 4 skipped. Not yet installed in a guest (no VM yet).</t>
         </is>
       </c>
     </row>
@@ -1545,7 +1545,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Workbench step B: drive = E: (Ravi 21-10: no 2 TB HDD; programs on C:, data on E:), E: measured Healthy, 1 GB write 30/15 MB/s; run folders on C:
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent-workbench/TRACKER.xlsx
+++ b/agent-workbench/TRACKER.xlsx
@@ -614,22 +614,23 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Decided 18-10-2026</t>
+          <t>Decided 21-10-2026</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Select after preflight</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Rule decided 18-10; measured 19-10: only C: (system) and E: (USB SanDisk SSD, kept for AVNI OS) are connected. 2 TB HDD absent -&gt; no drive chosen, nothing allocated | 20-10-2026 14:38 Ravi (phone ask-33c40ae475724999): 'I will plug in the 2 TB disk and allow Hyper-V'. 21-10-2026 17:4x: Hyper-V allowed and switched on; the 2 TB disk is still not connected (only C: and E:). No drive chosen, nothing allocated.</t>
+          <t>Rule decided 18-10; measured 19-10: only C: (system) and E: (USB SanDisk SSD, kept for AVNI OS) are connected. 2 TB HDD absent -&gt; no drive chosen, nothing allocated | 20-10-2026 14:38 Ravi (phone ask-33c40ae475724999): 'I will plug in the 2 TB disk and allow Hyper-V'. 21-10-2026 17:4x: Hyper-V allowed and switched on; the 2 TB disk is still not connected (only C: and E:). No drive chosen, nothing allocated. | 21-10-2026 18:2x RAVI: 'There will be no HDD 2 TB, 1 TB SSD is attached' + 'All programs stay on C only. Files from top priority to 1 which the program needs immediately stay on C. Others move to E.' DECISION: VM data (VHDX, checkpoints, ISO) on E:\AVNI-Workbench\ (E: = the detachable overflow drive by the C-to-E law; the Workbench is OFF by default and rebuildable from the ISO; C: has 58 GB free, below the 100 GB floor, so it cannot hold a VHDX). Programs (scripts, hands service, driver, run folders) stay on C:. AVNI_WORKBENCH_DATA (User) = %LOCALAPPDATA%\Avni\workbench+uns.</t>
         </is>
       </c>
     </row>
@@ -1389,27 +1390,27 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Evaluate the 2 TB HDD: health (SMART / Get-PhysicalDisk HealthStatus), free space, sequential and random performance (winsat disk or a 1 GB write/read timing) before it hosts the VHDX</t>
+          <t>Evaluate the Workbench drive (was: the 2 TB HDD; since 21-10-2026 the 1 TB SanDisk SSD E:): health, free space, timed 1 GB write/read before it hosts the VHDX</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4 min</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Local session, 10 min</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>19-10-2026: 2 TB HDD not connected to the PC (Get-PhysicalDisk shows only disk 0 NVMe + disk 1 SanDisk USB). Owner to plug it in | 21-10-2026 17:4x: still not connected (Get-Disk: 0 Samsung NVMe, 1 SanDisk USB).</t>
+          <t>19-10-2026: 2 TB HDD not connected to the PC (Get-PhysicalDisk shows only disk 0 NVMe + disk 1 SanDisk USB). Owner to plug it in | 21-10-2026 17:4x: still not connected (Get-Disk: 0 Samsung NVMe, 1 SanDisk USB). | 21-10-2026 18:29 MEASURED on E: (SanDisk Extreme 55DD, USB, SSD): HealthStatus Healthy, OperationalStatus OK, 931.5 GB / 839 GB free; 1 GB write with WriteThrough 68.5 s = 15 MB/s; 1 GB buffered write + Flush(true) 34.3 s = 30 MB/s; read of the same file 0.6 s = cache, not the disk. Reliability counters not exposed over USB. 30 MB/s is USB-2 class - the port/cable is being checked; the VM will work but Windows setup will be slow.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Workbench tracker: rows 5 (VM created), 6 (unattended setup prepared), 23 (isolation fixed and connected)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent-workbench/TRACKER.xlsx
+++ b/agent-workbench/TRACKER.xlsx
@@ -645,22 +645,22 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>1 session</t>
+          <t>35 s</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Local session, 10 min after decisions 3 and 4</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>host/New-Workbench.ps1 written, parse-checked only. Needs admin PowerShell on the PC.</t>
+          <t>host/New-Workbench.ps1 written, parse-checked only. Needs admin PowerShell on the PC. | 21-10-2026 18:46 INSTALLED on the PC (elevated New-Workbench.ps1 -VhdRoot E:\AVNI-Workbench\AVNI-VMs): Gen 2, dynamic VHDX 200 GB (0 GB on disk), memory 6 start / 2 min / 8 max GB dynamic, 4 vCPU, Secure Boot MicrosoftWindows, vTPM, Guest Service Interface on, adapter disconnected, AutomaticStartAction Nothing, State Off. Record %LOCALAPPDATA%\Avni\reports\workbench-create-21-10-2026_1845.json. No ISO attached yet (download in progress).</t>
         </is>
       </c>
     </row>
@@ -675,7 +675,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Windows setup needs a human at the console for the pilot. Steps printed by New-Workbench.ps1.</t>
+          <t>Windows setup needs a human at the console for the pilot. Steps printed by New-Workbench.ps1. | 21-10-2026: planned UNATTENDED, not by hand - autounattend.xml (local account, OOBE hidden, India time zone, UEFI partitions, image index 1) built into E:\AVNI-Workbench\iso\autounattend.iso (IMAPI2, no ADK); the guest account record stays on the PC only (%LOCALAPPDATA%\Avni\workbench\guest-account.json, never committed). Waits for the Windows ISO (8.2 GB) to finish.</t>
         </is>
       </c>
     </row>
@@ -1185,22 +1185,22 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2 sessions</t>
+          <t>2 runs</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Verify on PC</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Code done 18-10-2026: Extended Port ACLs deny RFC1918 + link-local + IPv6 ULA/link-local in and out; guest may reach the host (Default Switch gateway) ONLY for DNS (53) and hands-service replies, so host SMB/RDP/dev servers stay unreachable from the guest; public internet stays open; Connect refuses unless the deny rules are present and the gateway is unchanged. Test-WorkbenchIsolation.ps1 proves it over PowerShell Direct. UNVERIFIED on Hyper-V until the local session runs Apply then Test. Known: Default Switch subnet can change after a host reboot; re-Apply then.</t>
+          <t>Code done 18-10-2026: Extended Port ACLs deny RFC1918 + link-local + IPv6 ULA/link-local in and out; guest may reach the host (Default Switch gateway) ONLY for DNS (53) and hands-service replies, so host SMB/RDP/dev servers stay unreachable from the guest; public internet stays open; Connect refuses unless the deny rules are present and the gateway is unchanged. Test-WorkbenchIsolation.ps1 proves it over PowerShell Direct. UNVERIFIED on Hyper-V until the local session runs Apply then Test. Known: Default Switch subnet can change after a host reboot; re-Apply then. | 21-10-2026 18:49 first Connect FAILED: Hyper-V 0x800700B7 'Cannot create a file when that file already exists' - proven by an elevated test (18:5x) to be two Extended ACL rules with the same Direction+Weight on a live switch port; unique weights and IPv6 rules are accepted. Fix: Set-WorkbenchNetworkIsolation.ps1 1.1.0 gives every rule its own weight (Outbound deny 50-56, Inbound deny 40-46, host 60+, ExtraAllow 80+, Inbound hands 101) and refuses a plan with a duplicate before touching the switch. 18:58 run 2: Apply 21 rules read back, Show inventory MATCHES, Connect -&gt; SwitchName Default Switch, Connected True, VM Off. Behaviour proof (Test-WorkbenchIsolation.ps1) still pending until the guest runs.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Workbench step E: Windows installed unattended (checkpoint 'clean install'); step F first run NOT MEASURED - Default Switch gateway changed after a host boot, heal = re-apply
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent-workbench/TRACKER.xlsx
+++ b/agent-workbench/TRACKER.xlsx
@@ -675,22 +675,22 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>boot 20:16, answered 23:42</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Human clicks, ~40 min</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Windows setup needs a human at the console for the pilot. Steps printed by New-Workbench.ps1. | 21-10-2026: planned UNATTENDED, not by hand - autounattend.xml (local account, OOBE hidden, India time zone, UEFI partitions, image index 1) built into E:\AVNI-Workbench\iso\autounattend.iso (IMAPI2, no ADK); the guest account record stays on the PC only (%LOCALAPPDATA%\Avni\workbench\guest-account.json, never committed). Waits for the Windows ISO (8.2 GB) to finish.</t>
+          <t>Windows setup needs a human at the console for the pilot. Steps printed by New-Workbench.ps1. | 21-10-2026: planned UNATTENDED, not by hand - autounattend.xml (local account, OOBE hidden, India time zone, UEFI partitions, image index 1) built into E:\AVNI-Workbench\iso\autounattend.iso (IMAPI2, no ADK); the guest account record stays on the PC only (%LOCALAPPDATA%\Avni\workbench\guest-account.json, never committed). Waits for the Windows ISO (8.2 GB) to finish. | 21-10-2026 INSTALLED UNATTENDED: ISO (8,225,329,152 bytes, mounted + sources\install.wim checked) + autounattend.iso attached as DVDs, DVD first in the boot order, Start-VM 20:16, Enter sent through WMI Msvm_Keyboard.TypeKey for the 'Press any key' prompt (33 accepted), nobody clicked in vmconnect. Host power-off/boot at 22:36 switched the VM Off mid-way; minder restarted it 23:32; first-run 'Just a moment' until 23:42, then the guest answered PowerShell Direct as AVNI-WB01\agent, OOBEInProgress=0, explorer running. VHDX 16.6 GB. Checkpoint '21-10-2026 2342 clean install' created 23:43:56 (Workbench.ps1 -Action Checkpoint). Guest thumbnails via WMI GetVirtualSystemThumbnailImage in %LOCALAPPDATA%\Avni\workbench\runs\.</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>host/Workbench.ps1 parse-checked only.</t>
+          <t>host/Workbench.ps1 parse-checked only. | 21-10-2026 23:43 Checkpoint action USED on the PC: created and read back (Get-VMSnapshot). Status/Start/Ip/Connect still to be exercised.</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Code done 18-10-2026: Extended Port ACLs deny RFC1918 + link-local + IPv6 ULA/link-local in and out; guest may reach the host (Default Switch gateway) ONLY for DNS (53) and hands-service replies, so host SMB/RDP/dev servers stay unreachable from the guest; public internet stays open; Connect refuses unless the deny rules are present and the gateway is unchanged. Test-WorkbenchIsolation.ps1 proves it over PowerShell Direct. UNVERIFIED on Hyper-V until the local session runs Apply then Test. Known: Default Switch subnet can change after a host reboot; re-Apply then. | 21-10-2026 18:49 first Connect FAILED: Hyper-V 0x800700B7 'Cannot create a file when that file already exists' - proven by an elevated test (18:5x) to be two Extended ACL rules with the same Direction+Weight on a live switch port; unique weights and IPv6 rules are accepted. Fix: Set-WorkbenchNetworkIsolation.ps1 1.1.0 gives every rule its own weight (Outbound deny 50-56, Inbound deny 40-46, host 60+, ExtraAllow 80+, Inbound hands 101) and refuses a plan with a duplicate before touching the switch. 18:58 run 2: Apply 21 rules read back, Show inventory MATCHES, Connect -&gt; SwitchName Default Switch, Connected True, VM Off. Behaviour proof (Test-WorkbenchIsolation.ps1) still pending until the guest runs.</t>
+          <t>Code done 18-10-2026: Extended Port ACLs deny RFC1918 + link-local + IPv6 ULA/link-local in and out; guest may reach the host (Default Switch gateway) ONLY for DNS (53) and hands-service replies, so host SMB/RDP/dev servers stay unreachable from the guest; public internet stays open; Connect refuses unless the deny rules are present and the gateway is unchanged. Test-WorkbenchIsolation.ps1 proves it over PowerShell Direct. UNVERIFIED on Hyper-V until the local session runs Apply then Test. Known: Default Switch subnet can change after a host reboot; re-Apply then. | 21-10-2026 18:49 first Connect FAILED: Hyper-V 0x800700B7 'Cannot create a file when that file already exists' - proven by an elevated test (18:5x) to be two Extended ACL rules with the same Direction+Weight on a live switch port; unique weights and IPv6 rules are accepted. Fix: Set-WorkbenchNetworkIsolation.ps1 1.1.0 gives every rule its own weight (Outbound deny 50-56, Inbound deny 40-46, host 60+, ExtraAllow 80+, Inbound hands 101) and refuses a plan with a duplicate before touching the switch. 18:58 run 2: Apply 21 rules read back, Show inventory MATCHES, Connect -&gt; SwitchName Default Switch, Connected True, VM Off. Behaviour proof (Test-WorkbenchIsolation.ps1) still pending until the guest runs. | 21-10-2026 23:46 Test-WorkbenchIsolation.ps1 from inside the guest = NOT MEASURED (exit 2): every LAN and internet row failed instantly, DNS failed - the guest had NO internet, so blocked rows prove nothing. Cause measured on the host: a second host boot at 22:36 gave the Default Switch a NEW gateway 172.26.32.1/20 (rules built for 172.17.224.1); the new gateway sits inside the denied 172.16.0.0/12 range, so DHCP/DNS/NAT die. Heal = Apply again for the live gateway + ipconfig /renew in the guest; the minder now does this at every run.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Workbench step F: ISOLATION VERIFIED from inside the guest (22-10-2026 00:01) after the gateway heal
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent-workbench/TRACKER.xlsx
+++ b/agent-workbench/TRACKER.xlsx
@@ -930,7 +930,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>DECIDED (Architect 18-10-2026): guest-to-LAN block comes BEFORE the first network-connected guest boot. Mechanism: Hyper-V Extended Port ACLs on the VM adapter (host-enforced, the guest cannot lift them). Scripts: host/Set-WorkbenchNetworkIsolation.ps1 (Apply/Show/Remove/Connect/Disconnect) and host/Test-WorkbenchIsolation.ps1 (PowerShell Direct proof from inside the guest). New-Workbench now creates the adapter DISCONNECTED. Guest-only Git identity still owed.</t>
+          <t>DECIDED (Architect 18-10-2026): guest-to-LAN block comes BEFORE the first network-connected guest boot. Mechanism: Hyper-V Extended Port ACLs on the VM adapter (host-enforced, the guest cannot lift them). Scripts: host/Set-WorkbenchNetworkIsolation.ps1 (Apply/Show/Remove/Connect/Disconnect) and host/Test-WorkbenchIsolation.ps1 (PowerShell Direct proof from inside the guest). New-Workbench now creates the adapter DISCONNECTED. Guest-only Git identity still owed. | 22-10-2026: guest-only local account (record on the PC only), no host drive shares, office LAN blocked and VERIFIED from inside the guest; hands service bound to the host gateway only.</t>
         </is>
       </c>
     </row>
@@ -1185,12 +1185,12 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2 runs</t>
+          <t>3 runs</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Code done 18-10-2026: Extended Port ACLs deny RFC1918 + link-local + IPv6 ULA/link-local in and out; guest may reach the host (Default Switch gateway) ONLY for DNS (53) and hands-service replies, so host SMB/RDP/dev servers stay unreachable from the guest; public internet stays open; Connect refuses unless the deny rules are present and the gateway is unchanged. Test-WorkbenchIsolation.ps1 proves it over PowerShell Direct. UNVERIFIED on Hyper-V until the local session runs Apply then Test. Known: Default Switch subnet can change after a host reboot; re-Apply then. | 21-10-2026 18:49 first Connect FAILED: Hyper-V 0x800700B7 'Cannot create a file when that file already exists' - proven by an elevated test (18:5x) to be two Extended ACL rules with the same Direction+Weight on a live switch port; unique weights and IPv6 rules are accepted. Fix: Set-WorkbenchNetworkIsolation.ps1 1.1.0 gives every rule its own weight (Outbound deny 50-56, Inbound deny 40-46, host 60+, ExtraAllow 80+, Inbound hands 101) and refuses a plan with a duplicate before touching the switch. 18:58 run 2: Apply 21 rules read back, Show inventory MATCHES, Connect -&gt; SwitchName Default Switch, Connected True, VM Off. Behaviour proof (Test-WorkbenchIsolation.ps1) still pending until the guest runs. | 21-10-2026 23:46 Test-WorkbenchIsolation.ps1 from inside the guest = NOT MEASURED (exit 2): every LAN and internet row failed instantly, DNS failed - the guest had NO internet, so blocked rows prove nothing. Cause measured on the host: a second host boot at 22:36 gave the Default Switch a NEW gateway 172.26.32.1/20 (rules built for 172.17.224.1); the new gateway sits inside the denied 172.16.0.0/12 range, so DHCP/DNS/NAT die. Heal = Apply again for the live gateway + ipconfig /renew in the guest; the minder now does this at every run.</t>
+          <t>Code done 18-10-2026: Extended Port ACLs deny RFC1918 + link-local + IPv6 ULA/link-local in and out; guest may reach the host (Default Switch gateway) ONLY for DNS (53) and hands-service replies, so host SMB/RDP/dev servers stay unreachable from the guest; public internet stays open; Connect refuses unless the deny rules are present and the gateway is unchanged. Test-WorkbenchIsolation.ps1 proves it over PowerShell Direct. UNVERIFIED on Hyper-V until the local session runs Apply then Test. Known: Default Switch subnet can change after a host reboot; re-Apply then. | 21-10-2026 18:49 first Connect FAILED: Hyper-V 0x800700B7 'Cannot create a file when that file already exists' - proven by an elevated test (18:5x) to be two Extended ACL rules with the same Direction+Weight on a live switch port; unique weights and IPv6 rules are accepted. Fix: Set-WorkbenchNetworkIsolation.ps1 1.1.0 gives every rule its own weight (Outbound deny 50-56, Inbound deny 40-46, host 60+, ExtraAllow 80+, Inbound hands 101) and refuses a plan with a duplicate before touching the switch. 18:58 run 2: Apply 21 rules read back, Show inventory MATCHES, Connect -&gt; SwitchName Default Switch, Connected True, VM Off. Behaviour proof (Test-WorkbenchIsolation.ps1) still pending until the guest runs. | 21-10-2026 23:46 Test-WorkbenchIsolation.ps1 from inside the guest = NOT MEASURED (exit 2): every LAN and internet row failed instantly, DNS failed - the guest had NO internet, so blocked rows prove nothing. Cause measured on the host: a second host boot at 22:36 gave the Default Switch a NEW gateway 172.26.32.1/20 (rules built for 172.17.224.1); the new gateway sits inside the denied 172.16.0.0/12 range, so DHCP/DNS/NAT die. Heal = Apply again for the live gateway + ipconfig /renew in the guest; the minder now does this at every run. | 22-10-2026 00:01 ISOLATION VERIFIED (Test-WorkbenchIsolation.ps1 exit 0, from inside the guest over PowerShell Direct, after the heal: Disconnect, Apply for the live gateway 172.26.32.1, Show, Connect, ipconfig /renew): host ACL baseline 10 deny rules present; LAN 10.199.27.85 / 192.168.1.10 / 192.168.1.254 on TCP 445 + 3389 timed out 21-24 s each and ICMP no reply; host gateway 445/3389 no answer; internet 1.1.1.1 + 8.8.8.8 TCP 443 connected 0-0.1 s; DNS www.microsoft.com resolved 23.37.86.48. Report %LOCALAPPDATA%\Avni\reports\workbench-isolation-test-21-10-2026_2357.json. LESSON: this PC is powered off nightly and the Default Switch gateway changes on boot - run Disconnect/Apply/Connect (step-fg-minder3) before every use; a fixed-gateway internal NAT switch is the proper follow-up.</t>
         </is>
       </c>
     </row>

</xml_diff>